<commit_message>
refactor and add new feature
</commit_message>
<xml_diff>
--- a/CVB-Tabel.xlsx
+++ b/CVB-Tabel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ghanm\Documents\ILVO Projects\Drupal RekeningTool\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ghanm\Documents\ILVO Projects\Rekentool\livinglabs-tools\rundveeloket\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66B4AD13-76C2-4563-A882-3406ABAB992C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AB02F00-2674-40F8-9B7E-FC4F9BF988BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -612,7 +612,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -627,6 +627,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF222222"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -649,11 +655,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -934,7 +941,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G179"/>
+  <dimension ref="A1:G180"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47.85546875" customWidth="1"/>
@@ -5060,6 +5067,9 @@
         <v>1313.71325</v>
       </c>
     </row>
+    <row r="180" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B180" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>